<commit_message>
Cache daily screener results and link stock charts
</commit_message>
<xml_diff>
--- a/output/screening_result.xlsx
+++ b/output/screening_result.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,202 +429,202 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>candidate_level</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>candidate_score</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>市場</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>收盤價</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>MA20</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否站上 MA20</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>K 值</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>D 值</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Volume_MA5</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Volume_MA20</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Volume_MA40</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>放量倍數</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MACD_DIF</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MACD_Signal</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>MACD_Histogram</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>MACD_Histogram_前1日</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MACD_Histogram_前2日</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MACD_綠柱趨緩接近翻紅</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>是否符合 KD 區間</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>是否符合 RSI 區間</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>是否明顯放量</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MACD 是否綠柱趨緩接近翻紅</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>法人近 5 日是否合計買超</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>投信近 5 日是否買超</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>外資近 1 日買賣超張數</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>投信近 1 日買賣超張數</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>自營商近 1 日買賣超張數</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>三大法人近 1 日合計買賣超張數</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>外資近 5 日買賣超張數</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>投信近 5 日買賣超張數</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>自營商近 5 日買賣超張數</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>三大法人近 5 日合計買賣超張數</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>外資近 20 日買賣超張數</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>投信近 20 日買賣超張數</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>自營商近 20 日買賣超張數</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>三大法人近 20 日合計買賣超張數</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>最後更新日期</t>
         </is>
@@ -673,19 +685,19 @@
         <v>1.839402433396137</v>
       </c>
       <c r="P2" t="n">
-        <v>0.05707517759306668</v>
+        <v>0.0570751775930666</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.002957888560102742</v>
+        <v>-0.0029578885601027</v>
       </c>
       <c r="R2" t="n">
-        <v>0.06003306615316942</v>
+        <v>0.0600330661531694</v>
       </c>
       <c r="S2" t="n">
-        <v>0.08140312991042646</v>
+        <v>0.08140312991042641</v>
       </c>
       <c r="T2" t="n">
-        <v>0.1191330164089761</v>
+        <v>0.119133016408976</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -819,19 +831,19 @@
         <v>1.580724998413493</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.1808840313655367</v>
+        <v>-0.1808840313655366</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.1408225222788201</v>
+        <v>-0.14082252227882</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.04006150908671657</v>
+        <v>-0.0400615090867165</v>
       </c>
       <c r="S3" t="n">
-        <v>-0.05093762199336851</v>
+        <v>-0.0509376219933685</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.05194541608982742</v>
+        <v>-0.0519454160898274</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -971,13 +983,13 @@
         <v>-0.4985450554719721</v>
       </c>
       <c r="R4" t="n">
-        <v>0.04336846687852813</v>
+        <v>0.0433684668785281</v>
       </c>
       <c r="S4" t="n">
-        <v>0.04526563362469704</v>
+        <v>0.045265633624697</v>
       </c>
       <c r="T4" t="n">
-        <v>0.05191589189844181</v>
+        <v>0.0519158918984418</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -1117,13 +1129,13 @@
         <v>-0.7662871133930196</v>
       </c>
       <c r="R5" t="n">
-        <v>0.05304759902012179</v>
+        <v>0.0530475990201217</v>
       </c>
       <c r="S5" t="n">
-        <v>0.05140381760834511</v>
+        <v>0.0514038176083451</v>
       </c>
       <c r="T5" t="n">
-        <v>0.06091183394929145</v>
+        <v>0.0609118339492914</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -1260,16 +1272,16 @@
         <v>-0.038684783307672</v>
       </c>
       <c r="Q6" t="n">
-        <v>-0.07277598983752707</v>
+        <v>-0.07277598983752701</v>
       </c>
       <c r="R6" t="n">
-        <v>0.03409120652985508</v>
+        <v>0.034091206529855</v>
       </c>
       <c r="S6" t="n">
-        <v>0.03959072830204988</v>
+        <v>0.0395907283020498</v>
       </c>
       <c r="T6" t="n">
-        <v>0.03910897843283044</v>
+        <v>0.0391089784328304</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1412,10 +1424,10 @@
         <v>-0.0249666651297922</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.02023013043446435</v>
+        <v>-0.0202301304344643</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.008345501526961507</v>
+        <v>-0.0083455015269615</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -1555,7 +1567,7 @@
         <v>-0.3800329123209913</v>
       </c>
       <c r="R8" t="n">
-        <v>-0.06135081899517369</v>
+        <v>-0.0613508189951736</v>
       </c>
       <c r="S8" t="n">
         <v>-0.09689548365965001</v>
@@ -1695,19 +1707,19 @@
         <v>1.798804727870702</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.2419575748652605</v>
+        <v>-0.2419575748652604</v>
       </c>
       <c r="Q9" t="n">
-        <v>-0.1266850911670767</v>
+        <v>-0.1266850911670766</v>
       </c>
       <c r="R9" t="n">
         <v>-0.1152724836981838</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.09662280170647791</v>
+        <v>-0.0966228017064779</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.01663634277134032</v>
+        <v>-0.0166363427713403</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -1841,19 +1853,19 @@
         <v>1.7832781618118</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.005917047706663681</v>
+        <v>-0.0059170477066636</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.07419920651975694</v>
+        <v>-0.07419920651975689</v>
       </c>
       <c r="R10" t="n">
-        <v>0.06828215881309325</v>
+        <v>0.0682821588130932</v>
       </c>
       <c r="S10" t="n">
-        <v>0.08930145589692245</v>
+        <v>0.0893014558969224</v>
       </c>
       <c r="T10" t="n">
-        <v>0.1217865254905505</v>
+        <v>0.1217865254905504</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1996,7 +2008,7 @@
         <v>0.3776729282985334</v>
       </c>
       <c r="S11" t="n">
-        <v>0.4825700324428605</v>
+        <v>0.4825700324428604</v>
       </c>
       <c r="T11" t="n">
         <v>0.662287037074081</v>
@@ -2136,7 +2148,7 @@
         <v>0.3598539212373666</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2020636183624591</v>
+        <v>0.202063618362459</v>
       </c>
       <c r="R12" t="n">
         <v>0.1577903028749075</v>
@@ -2282,16 +2294,16 @@
         <v>-0.3881676954178754</v>
       </c>
       <c r="Q13" t="n">
-        <v>-0.431135773024979</v>
+        <v>-0.4311357730249789</v>
       </c>
       <c r="R13" t="n">
-        <v>0.04296807760710353</v>
+        <v>0.0429680776071035</v>
       </c>
       <c r="S13" t="n">
-        <v>0.00374273470610087</v>
+        <v>0.0037427347061008</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.02217975833307273</v>
+        <v>-0.0221797583330727</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -2425,19 +2437,19 @@
         <v>1.635955388215924</v>
       </c>
       <c r="P14" t="n">
-        <v>0.04252266497129398</v>
+        <v>0.0425226649712939</v>
       </c>
       <c r="Q14" t="n">
         <v>0.1163449674426191</v>
       </c>
       <c r="R14" t="n">
-        <v>-0.07382230247132515</v>
+        <v>-0.0738223024713251</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.04122709533962188</v>
+        <v>-0.0412270953396218</v>
       </c>
       <c r="T14" t="n">
-        <v>0.002082373979241658</v>
+        <v>0.0020823739792416</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
@@ -2580,10 +2592,10 @@
         <v>-0.06671035967326749</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.05169010730895907</v>
+        <v>-0.051690107308959</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.01237562072793957</v>
+        <v>-0.0123756207279395</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
@@ -2696,7 +2708,7 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>30.18586796019645</v>
+        <v>30.18586796019646</v>
       </c>
       <c r="J16" t="n">
         <v>45.14705019354905</v>
@@ -2726,10 +2738,10 @@
         <v>-0.2046288617528741</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.05205642433026325</v>
+        <v>-0.0520564243302632</v>
       </c>
       <c r="T16" t="n">
-        <v>0.1062483856006611</v>
+        <v>0.106248385600661</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -2860,7 +2872,7 @@
         <v>5389496.05</v>
       </c>
       <c r="O17" t="n">
-        <v>1.896273292690601</v>
+        <v>1.896273292690602</v>
       </c>
       <c r="P17" t="n">
         <v>0.4038925206493076</v>
@@ -2872,10 +2884,10 @@
         <v>0.116457645451703</v>
       </c>
       <c r="S17" t="n">
-        <v>0.4941181782478166</v>
+        <v>0.4941181782478165</v>
       </c>
       <c r="T17" t="n">
-        <v>0.9293924714675723</v>
+        <v>0.9293924714675724</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -2988,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>30.53242543371862</v>
+        <v>30.53242543371863</v>
       </c>
       <c r="J18" t="n">
         <v>41.61517745627029</v>
@@ -3015,13 +3027,13 @@
         <v>-0.4106534675819211</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.08040273606741488</v>
+        <v>-0.0804027360674148</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.04073207890847924</v>
+        <v>-0.0407320789084792</v>
       </c>
       <c r="T18" t="n">
-        <v>0.03164810210110147</v>
+        <v>0.0316481021011014</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
@@ -3161,13 +3173,13 @@
         <v>-0.3359433016543629</v>
       </c>
       <c r="R19" t="n">
-        <v>0.06458651840347929</v>
+        <v>0.0645865184034792</v>
       </c>
       <c r="S19" t="n">
-        <v>0.06947599190700904</v>
+        <v>0.069475991907009</v>
       </c>
       <c r="T19" t="n">
-        <v>0.09695122744569268</v>
+        <v>0.09695122744569259</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
@@ -3307,13 +3319,13 @@
         <v>0.256726040843972</v>
       </c>
       <c r="R20" t="n">
-        <v>-0.04401885643618519</v>
+        <v>-0.0440188564361851</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.01763998701829256</v>
+        <v>-0.0176399870182925</v>
       </c>
       <c r="T20" t="n">
-        <v>0.01184571612104895</v>
+        <v>0.0118457161210489</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -3447,19 +3459,19 @@
         <v>1.525494998136593</v>
       </c>
       <c r="P21" t="n">
-        <v>-0.06302702848723207</v>
+        <v>-0.063027028487232</v>
       </c>
       <c r="Q21" t="n">
-        <v>-0.03444490503477615</v>
+        <v>-0.0344449050347761</v>
       </c>
       <c r="R21" t="n">
-        <v>-0.02858212345245592</v>
+        <v>-0.0285821234524559</v>
       </c>
       <c r="S21" t="n">
-        <v>0.002827214278937951</v>
+        <v>0.0028272142789379</v>
       </c>
       <c r="T21" t="n">
-        <v>0.01440908807375371</v>
+        <v>0.0144090880737537</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -3596,16 +3608,16 @@
         <v>-0.1481337758828047</v>
       </c>
       <c r="Q22" t="n">
-        <v>-0.1451000600982614</v>
+        <v>-0.1451000600982613</v>
       </c>
       <c r="R22" t="n">
-        <v>-0.003033715784543367</v>
+        <v>-0.0030337157845433</v>
       </c>
       <c r="S22" t="n">
-        <v>-0.006370086530677693</v>
+        <v>-0.0063700865306776</v>
       </c>
       <c r="T22" t="n">
-        <v>-0.009060828894512735</v>
+        <v>-0.0090608288945127</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
@@ -3745,13 +3757,13 @@
         <v>-1.312189918065065</v>
       </c>
       <c r="R23" t="n">
-        <v>0.3244853267880852</v>
+        <v>0.3244853267880851</v>
       </c>
       <c r="S23" t="n">
         <v>0.3180542302507319</v>
       </c>
       <c r="T23" t="n">
-        <v>0.3014591542416836</v>
+        <v>0.3014591542416835</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
@@ -3891,13 +3903,13 @@
         <v>-0.2724307945518312</v>
       </c>
       <c r="R24" t="n">
-        <v>-0.02852609044847937</v>
+        <v>-0.0285260904484793</v>
       </c>
       <c r="S24" t="n">
-        <v>-0.01496776097232111</v>
+        <v>-0.0149677609723211</v>
       </c>
       <c r="T24" t="n">
-        <v>-0.008588931923730447</v>
+        <v>-0.008588931923730401</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -4031,19 +4043,19 @@
         <v>1.003173868321978</v>
       </c>
       <c r="P25" t="n">
-        <v>-0.06332718323102426</v>
+        <v>-0.06332718323102419</v>
       </c>
       <c r="Q25" t="n">
-        <v>-0.03359213917101796</v>
+        <v>-0.0335921391710179</v>
       </c>
       <c r="R25" t="n">
         <v>-0.0297350440600063</v>
       </c>
       <c r="S25" t="n">
-        <v>-0.02997532303726926</v>
+        <v>-0.0299753230372692</v>
       </c>
       <c r="T25" t="n">
-        <v>-0.05292571016015371</v>
+        <v>-0.0529257101601537</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
@@ -4177,19 +4189,19 @@
         <v>0.96482269131437</v>
       </c>
       <c r="P26" t="n">
-        <v>-0.1351788962546561</v>
+        <v>-0.135178896254656</v>
       </c>
       <c r="Q26" t="n">
         <v>-0.1280823181746952</v>
       </c>
       <c r="R26" t="n">
-        <v>-0.007096578079960836</v>
+        <v>-0.0070965780799608</v>
       </c>
       <c r="S26" t="n">
-        <v>-0.02687530782058334</v>
+        <v>-0.0268753078205833</v>
       </c>
       <c r="T26" t="n">
-        <v>-0.04416464935125755</v>
+        <v>-0.0441646493512575</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
@@ -4320,22 +4332,22 @@
         <v>1125916.225</v>
       </c>
       <c r="O27" t="n">
-        <v>0.9105588305876801</v>
+        <v>0.9105588305876799</v>
       </c>
       <c r="P27" t="n">
         <v>-0.0184294891631076</v>
       </c>
       <c r="Q27" t="n">
-        <v>-0.02050138599078901</v>
+        <v>-0.020501385990789</v>
       </c>
       <c r="R27" t="n">
-        <v>0.00207189682768141</v>
+        <v>0.0020718968276814</v>
       </c>
       <c r="S27" t="n">
-        <v>0.002602296497784571</v>
+        <v>0.0026022964977845</v>
       </c>
       <c r="T27" t="n">
-        <v>0.003536614594513193</v>
+        <v>0.0035366145945131</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
@@ -4469,19 +4481,19 @@
         <v>0.3081990758454248</v>
       </c>
       <c r="P28" t="n">
-        <v>-0.03334931484251857</v>
+        <v>-0.0333493148425185</v>
       </c>
       <c r="Q28" t="n">
-        <v>-0.01046773277712322</v>
+        <v>-0.0104677327771232</v>
       </c>
       <c r="R28" t="n">
-        <v>-0.02288158206539535</v>
+        <v>-0.0228815820653953</v>
       </c>
       <c r="S28" t="n">
-        <v>-0.02567799944667791</v>
+        <v>-0.0256779994466779</v>
       </c>
       <c r="T28" t="n">
-        <v>-0.02690468446860406</v>
+        <v>-0.026904684468604</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -4588,7 +4600,7 @@
         <v>27.5</v>
       </c>
       <c r="G29" t="n">
-        <v>28.71749992370605</v>
+        <v>28.71749992370606</v>
       </c>
       <c r="H29" t="b">
         <v>0</v>
@@ -4615,7 +4627,7 @@
         <v>2.125165839050832</v>
       </c>
       <c r="P29" t="n">
-        <v>-0.1101141161981012</v>
+        <v>-0.1101141161981011</v>
       </c>
       <c r="Q29" t="n">
         <v>0.114495724853119</v>
@@ -4904,7 +4916,7 @@
         <v>158878.775</v>
       </c>
       <c r="O31" t="n">
-        <v>1.837621951233754</v>
+        <v>1.837621951233753</v>
       </c>
       <c r="P31" t="n">
         <v>-0.303341141391666</v>
@@ -4913,13 +4925,13 @@
         <v>-0.5186348610355919</v>
       </c>
       <c r="R31" t="n">
-        <v>0.2152937196439259</v>
+        <v>0.2152937196439258</v>
       </c>
       <c r="S31" t="n">
         <v>0.2587159426150786</v>
       </c>
       <c r="T31" t="n">
-        <v>0.2485007574791648</v>
+        <v>0.2485007574791647</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
@@ -5059,13 +5071,13 @@
         <v>-0.1667161311207628</v>
       </c>
       <c r="R32" t="n">
-        <v>-0.03438024783712951</v>
+        <v>-0.0343802478371295</v>
       </c>
       <c r="S32" t="n">
-        <v>-0.07952984104989819</v>
+        <v>-0.0795298410498981</v>
       </c>
       <c r="T32" t="n">
-        <v>-0.09679417573719046</v>
+        <v>-0.0967941757371904</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
@@ -5351,13 +5363,13 @@
         <v>-0.0903966745737473</v>
       </c>
       <c r="R34" t="n">
-        <v>-0.03258721900541321</v>
+        <v>-0.0325872190054132</v>
       </c>
       <c r="S34" t="n">
-        <v>-0.001717367964322009</v>
+        <v>-0.001717367964322</v>
       </c>
       <c r="T34" t="n">
-        <v>0.00814664426163085</v>
+        <v>0.0081466442616308</v>
       </c>
       <c r="U34" t="inlineStr">
         <is>
@@ -5497,13 +5509,13 @@
         <v>-0.2935732383990579</v>
       </c>
       <c r="R35" t="n">
-        <v>0.04794177147055367</v>
+        <v>0.0479417714705536</v>
       </c>
       <c r="S35" t="n">
-        <v>0.04320541528264987</v>
+        <v>0.0432054152826498</v>
       </c>
       <c r="T35" t="n">
-        <v>0.05175250589301905</v>
+        <v>0.051752505893019</v>
       </c>
       <c r="U35" t="inlineStr">
         <is>
@@ -5643,13 +5655,13 @@
         <v>-0.9542266912467944</v>
       </c>
       <c r="R36" t="n">
-        <v>-0.08771832645632649</v>
+        <v>-0.08771832645632641</v>
       </c>
       <c r="S36" t="n">
         <v>-0.0869277373098295</v>
       </c>
       <c r="T36" t="n">
-        <v>-0.07501743440886655</v>
+        <v>-0.0750174344088665</v>
       </c>
       <c r="U36" t="inlineStr">
         <is>
@@ -5792,10 +5804,10 @@
         <v>-0.9152645595746156</v>
       </c>
       <c r="S37" t="n">
-        <v>-0.9486018252643413</v>
+        <v>-0.9486018252643412</v>
       </c>
       <c r="T37" t="n">
-        <v>-0.2695243893553894</v>
+        <v>-0.2695243893553893</v>
       </c>
       <c r="U37" t="inlineStr">
         <is>
@@ -5857,7 +5869,7 @@
         <v>-561.461</v>
       </c>
       <c r="AJ37" t="n">
-        <v>-922.3249999999999</v>
+        <v>-922.325</v>
       </c>
       <c r="AK37" t="n">
         <v>0</v>
@@ -5929,16 +5941,16 @@
         <v>1.523473055739829</v>
       </c>
       <c r="P38" t="n">
-        <v>-0.002821873993433144</v>
+        <v>-0.0028218739934331</v>
       </c>
       <c r="Q38" t="n">
-        <v>-0.06410956955032149</v>
+        <v>-0.0641095695503214</v>
       </c>
       <c r="R38" t="n">
-        <v>0.06128769555688834</v>
+        <v>0.0612876955568883</v>
       </c>
       <c r="S38" t="n">
-        <v>0.09929104468963655</v>
+        <v>0.0992910446896365</v>
       </c>
       <c r="T38" t="n">
         <v>0.1476838546539809</v>
@@ -6224,16 +6236,16 @@
         <v>-0.2269263504303893</v>
       </c>
       <c r="Q40" t="n">
-        <v>-0.2314013296597059</v>
+        <v>-0.2314013296597058</v>
       </c>
       <c r="R40" t="n">
-        <v>0.004474979229316528</v>
+        <v>0.0044749792293165</v>
       </c>
       <c r="S40" t="n">
-        <v>-0.02490320946406871</v>
+        <v>-0.0249032094640687</v>
       </c>
       <c r="T40" t="n">
-        <v>-0.03576408482575447</v>
+        <v>-0.0357640848257544</v>
       </c>
       <c r="U40" t="inlineStr">
         <is>
@@ -6367,19 +6379,19 @@
         <v>1.43446646883085</v>
       </c>
       <c r="P41" t="n">
-        <v>-0.01315781132596072</v>
+        <v>-0.0131578113259607</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.2489182445671212</v>
+        <v>0.2489182445671211</v>
       </c>
       <c r="R41" t="n">
         <v>-0.2620760558930819</v>
       </c>
       <c r="S41" t="n">
-        <v>-0.1453064809411631</v>
+        <v>-0.145306480941163</v>
       </c>
       <c r="T41" t="n">
-        <v>-0.04815400939448922</v>
+        <v>-0.0481540093944892</v>
       </c>
       <c r="U41" t="inlineStr">
         <is>
@@ -6516,7 +6528,7 @@
         <v>-0.260311710181341</v>
       </c>
       <c r="Q42" t="n">
-        <v>-0.4066925966822941</v>
+        <v>-0.406692596682294</v>
       </c>
       <c r="R42" t="n">
         <v>0.146380886500953</v>
@@ -6525,7 +6537,7 @@
         <v>0.2071291220801476</v>
       </c>
       <c r="T42" t="n">
-        <v>0.242265375992006</v>
+        <v>0.2422653759920059</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
@@ -6659,10 +6671,10 @@
         <v>1.414631500155851</v>
       </c>
       <c r="P43" t="n">
-        <v>-0.09520171982933334</v>
+        <v>-0.0952017198293333</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.2468707643551459</v>
+        <v>0.2468707643551458</v>
       </c>
       <c r="R43" t="n">
         <v>-0.3420724841844792</v>
@@ -6671,7 +6683,7 @@
         <v>-0.3131464164646977</v>
       </c>
       <c r="T43" t="n">
-        <v>-0.1947314191951318</v>
+        <v>-0.1947314191951317</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
@@ -6802,7 +6814,7 @@
         <v>43862</v>
       </c>
       <c r="O44" t="n">
-        <v>1.381644559510172</v>
+        <v>1.381644559510173</v>
       </c>
       <c r="P44" t="n">
         <v>-1.644154325531758</v>
@@ -6957,13 +6969,13 @@
         <v>-0.6887826229136117</v>
       </c>
       <c r="R45" t="n">
-        <v>0.09018362819220516</v>
+        <v>0.0901836281922051</v>
       </c>
       <c r="S45" t="n">
-        <v>0.09022867952628122</v>
+        <v>0.09022867952628121</v>
       </c>
       <c r="T45" t="n">
-        <v>0.1134644690749076</v>
+        <v>0.1134644690749075</v>
       </c>
       <c r="U45" t="inlineStr">
         <is>
@@ -7097,19 +7109,19 @@
         <v>1.340713262650776</v>
       </c>
       <c r="P46" t="n">
-        <v>0.1678286692455693</v>
+        <v>0.1678286692455692</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.1847590204761862</v>
+        <v>0.1847590204761861</v>
       </c>
       <c r="R46" t="n">
-        <v>-0.0169303512306169</v>
+        <v>-0.0169303512306168</v>
       </c>
       <c r="S46" t="n">
-        <v>0.01600186697586498</v>
+        <v>0.0160018669758649</v>
       </c>
       <c r="T46" t="n">
-        <v>0.07463827441465035</v>
+        <v>0.0746382744146503</v>
       </c>
       <c r="U46" t="inlineStr">
         <is>
@@ -7243,16 +7255,16 @@
         <v>1.325407881462036</v>
       </c>
       <c r="P47" t="n">
-        <v>0.009704539192306072</v>
+        <v>0.009704539192306001</v>
       </c>
       <c r="Q47" t="n">
-        <v>-0.02457551877163998</v>
+        <v>-0.0245755187716399</v>
       </c>
       <c r="R47" t="n">
-        <v>0.03428005796394605</v>
+        <v>0.034280057963946</v>
       </c>
       <c r="S47" t="n">
-        <v>0.07140723864166555</v>
+        <v>0.0714072386416655</v>
       </c>
       <c r="T47" t="n">
         <v>0.1200608172714291</v>
@@ -7395,10 +7407,10 @@
         <v>-0.7451304069886938</v>
       </c>
       <c r="R48" t="n">
-        <v>0.02875490875487763</v>
+        <v>0.0287549087548776</v>
       </c>
       <c r="S48" t="n">
-        <v>0.05789699160078599</v>
+        <v>0.0578969916007859</v>
       </c>
       <c r="T48" t="n">
         <v>0.1104923900681894</v>
@@ -7541,13 +7553,13 @@
         <v>-1.744359638676258</v>
       </c>
       <c r="R49" t="n">
-        <v>-0.08298486444700637</v>
+        <v>-0.0829848644470063</v>
       </c>
       <c r="S49" t="n">
-        <v>-0.1355131032599302</v>
+        <v>-0.1355131032599301</v>
       </c>
       <c r="T49" t="n">
-        <v>-0.1930966195847468</v>
+        <v>-0.1930966195847467</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
@@ -7681,19 +7693,19 @@
         <v>1.28115306772091</v>
       </c>
       <c r="P50" t="n">
-        <v>-0.3888881856668434</v>
+        <v>-0.3888881856668433</v>
       </c>
       <c r="Q50" t="n">
         <v>-0.3328958859890168</v>
       </c>
       <c r="R50" t="n">
-        <v>-0.05599229967782654</v>
+        <v>-0.0559922996778265</v>
       </c>
       <c r="S50" t="n">
-        <v>-0.06614592339677605</v>
+        <v>-0.066145923396776</v>
       </c>
       <c r="T50" t="n">
-        <v>-0.07217485039420335</v>
+        <v>-0.07217485039420329</v>
       </c>
       <c r="U50" t="inlineStr">
         <is>
@@ -7827,19 +7839,19 @@
         <v>1.240810864329066</v>
       </c>
       <c r="P51" t="n">
-        <v>-0.05570595249982624</v>
+        <v>-0.0557059524998262</v>
       </c>
       <c r="Q51" t="n">
         <v>-0.0742800960870406</v>
       </c>
       <c r="R51" t="n">
-        <v>0.01857414358721436</v>
+        <v>0.0185741435872143</v>
       </c>
       <c r="S51" t="n">
-        <v>0.01668428170683153</v>
+        <v>0.0166842817068315</v>
       </c>
       <c r="T51" t="n">
-        <v>-0.01712381353649825</v>
+        <v>-0.0171238135364982</v>
       </c>
       <c r="U51" t="inlineStr">
         <is>
@@ -7979,13 +7991,13 @@
         <v>-0.2790708529521356</v>
       </c>
       <c r="R52" t="n">
-        <v>-0.03854497710318128</v>
+        <v>-0.0385449771031812</v>
       </c>
       <c r="S52" t="n">
-        <v>-0.002399427678093979</v>
+        <v>-0.0023994276780939</v>
       </c>
       <c r="T52" t="n">
-        <v>0.02375228502969762</v>
+        <v>0.0237522850296976</v>
       </c>
       <c r="U52" t="inlineStr">
         <is>
@@ -8044,7 +8056,7 @@
         <v>-2.344</v>
       </c>
       <c r="AI52" t="n">
-        <v>0.1560000000000006</v>
+        <v>0.1560000000000005</v>
       </c>
       <c r="AJ52" t="n">
         <v>31.86</v>
@@ -8119,16 +8131,16 @@
         <v>1.198011196029598</v>
       </c>
       <c r="P53" t="n">
-        <v>0.004120599986180196</v>
+        <v>0.0041205999861801</v>
       </c>
       <c r="Q53" t="n">
-        <v>-0.01432192550611949</v>
+        <v>-0.0143219255061194</v>
       </c>
       <c r="R53" t="n">
-        <v>0.01844252549229968</v>
+        <v>0.0184425254922996</v>
       </c>
       <c r="S53" t="n">
-        <v>0.09111258937696368</v>
+        <v>0.09111258937696361</v>
       </c>
       <c r="T53" t="n">
         <v>0.1488003391996831</v>
@@ -8274,7 +8286,7 @@
         <v>-0.4089015225913984</v>
       </c>
       <c r="S54" t="n">
-        <v>-0.3406516827308617</v>
+        <v>-0.3406516827308616</v>
       </c>
       <c r="T54" t="n">
         <v>-0.2072290987675836</v>
@@ -8411,19 +8423,19 @@
         <v>0.9495123450491636</v>
       </c>
       <c r="P55" t="n">
-        <v>-0.9082974689741405</v>
+        <v>-0.9082974689741404</v>
       </c>
       <c r="Q55" t="n">
         <v>-0.8889721184411055</v>
       </c>
       <c r="R55" t="n">
-        <v>-0.01932535053303508</v>
+        <v>-0.019325350533035</v>
       </c>
       <c r="S55" t="n">
-        <v>-0.06494275914383318</v>
+        <v>-0.0649427591438331</v>
       </c>
       <c r="T55" t="n">
-        <v>-0.08888607844110752</v>
+        <v>-0.0888860784411075</v>
       </c>
       <c r="U55" t="inlineStr">
         <is>
@@ -8563,10 +8575,10 @@
         <v>-0.6609626253823604</v>
       </c>
       <c r="R56" t="n">
-        <v>0.06813888047874861</v>
+        <v>0.0681388804787486</v>
       </c>
       <c r="S56" t="n">
-        <v>0.1008923160634631</v>
+        <v>0.100892316063463</v>
       </c>
       <c r="T56" t="n">
         <v>0.124027458424071</v>
@@ -8852,7 +8864,7 @@
         <v>0.4437671585590763</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.1677740635469122</v>
+        <v>0.1677740635469121</v>
       </c>
       <c r="R58" t="n">
         <v>0.2759930950121642</v>
@@ -8977,7 +8989,7 @@
         <v>39.19161417957683</v>
       </c>
       <c r="J59" t="n">
-        <v>28.48365925360274</v>
+        <v>28.48365925360273</v>
       </c>
       <c r="K59" t="n">
         <v>24.56157188356397</v>
@@ -9007,7 +9019,7 @@
         <v>-0.1364299700650431</v>
       </c>
       <c r="T59" t="n">
-        <v>-0.2232740689086299</v>
+        <v>-0.2232740689086298</v>
       </c>
       <c r="U59" t="inlineStr">
         <is>
@@ -9257,7 +9269,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>99.19999694824219</v>
+        <v>99.1999969482422</v>
       </c>
       <c r="G61" t="n">
         <v>99.53500022888184</v>
@@ -9296,10 +9308,10 @@
         <v>-0.1487675186313835</v>
       </c>
       <c r="S61" t="n">
-        <v>-0.08198202307414848</v>
+        <v>-0.0819820230741484</v>
       </c>
       <c r="T61" t="n">
-        <v>-0.04213063596094624</v>
+        <v>-0.0421306359609462</v>
       </c>
       <c r="U61" t="inlineStr">
         <is>
@@ -9436,16 +9448,16 @@
         <v>0.2013740750501469</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.1220078887518429</v>
+        <v>0.1220078887518428</v>
       </c>
       <c r="R62" t="n">
-        <v>0.07936618629830404</v>
+        <v>0.079366186298304</v>
       </c>
       <c r="S62" t="n">
         <v>-0.1137881662573722</v>
       </c>
       <c r="T62" t="n">
-        <v>-0.1033808123851388</v>
+        <v>-0.1033808123851387</v>
       </c>
       <c r="U62" t="inlineStr">
         <is>
@@ -9585,13 +9597,13 @@
         <v>-1.04579931371177</v>
       </c>
       <c r="R63" t="n">
-        <v>-0.03020957886800346</v>
+        <v>-0.0302095788680034</v>
       </c>
       <c r="S63" t="n">
-        <v>-0.1238112854771514</v>
+        <v>-0.1238112854771513</v>
       </c>
       <c r="T63" t="n">
-        <v>-0.1458734728691891</v>
+        <v>-0.145873472869189</v>
       </c>
       <c r="U63" t="inlineStr">
         <is>
@@ -9704,7 +9716,7 @@
         <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>13.27282771460793</v>
+        <v>13.27282771460794</v>
       </c>
       <c r="J64" t="n">
         <v>15.72798670235252</v>
@@ -9731,13 +9743,13 @@
         <v>-0.5193139278924654</v>
       </c>
       <c r="R64" t="n">
-        <v>-0.06815659551818243</v>
+        <v>-0.0681565955181824</v>
       </c>
       <c r="S64" t="n">
-        <v>-0.06804932552052112</v>
+        <v>-0.06804932552052111</v>
       </c>
       <c r="T64" t="n">
-        <v>-0.02942642255870948</v>
+        <v>-0.0294264225587094</v>
       </c>
       <c r="U64" t="inlineStr">
         <is>
@@ -9871,19 +9883,19 @@
         <v>1.37898931550765</v>
       </c>
       <c r="P65" t="n">
-        <v>-0.01453945324268346</v>
+        <v>-0.0145394532426834</v>
       </c>
       <c r="Q65" t="n">
-        <v>-0.08802936976482212</v>
+        <v>-0.0880293697648221</v>
       </c>
       <c r="R65" t="n">
-        <v>0.07348991652213865</v>
+        <v>0.0734899165221386</v>
       </c>
       <c r="S65" t="n">
-        <v>0.07750027075102853</v>
+        <v>0.0775002707510285</v>
       </c>
       <c r="T65" t="n">
-        <v>0.06878276824500457</v>
+        <v>0.0687827682450045</v>
       </c>
       <c r="U65" t="inlineStr">
         <is>
@@ -10023,10 +10035,10 @@
         <v>-0.5122927222630316</v>
       </c>
       <c r="R66" t="n">
-        <v>-0.1334825158475135</v>
+        <v>-0.1334825158475134</v>
       </c>
       <c r="S66" t="n">
-        <v>-0.09961932821432845</v>
+        <v>-0.0996193282143284</v>
       </c>
       <c r="T66" t="n">
         <v>-0.0302942136827089</v>
@@ -10172,7 +10184,7 @@
         <v>-0.3080662720564682</v>
       </c>
       <c r="S67" t="n">
-        <v>-0.2965847479391686</v>
+        <v>-0.2965847479391685</v>
       </c>
       <c r="T67" t="n">
         <v>-0.2093121514365122</v>
@@ -10318,7 +10330,7 @@
         <v>0.2702761204300148</v>
       </c>
       <c r="S68" t="n">
-        <v>0.2798058129214102</v>
+        <v>0.2798058129214101</v>
       </c>
       <c r="T68" t="n">
         <v>0.2138849747076076</v>
@@ -10437,7 +10449,7 @@
         <v>29.00532850935085</v>
       </c>
       <c r="J69" t="n">
-        <v>24.62943694085086</v>
+        <v>24.62943694085087</v>
       </c>
       <c r="K69" t="n">
         <v>42.40217427289991</v>
@@ -10458,16 +10470,16 @@
         <v>-0.2438031422359863</v>
       </c>
       <c r="Q69" t="n">
-        <v>-0.2289982268268628</v>
+        <v>-0.2289982268268627</v>
       </c>
       <c r="R69" t="n">
-        <v>-0.01480491540912354</v>
+        <v>-0.0148049154091235</v>
       </c>
       <c r="S69" t="n">
-        <v>-0.02873366415693418</v>
+        <v>-0.0287336641569341</v>
       </c>
       <c r="T69" t="n">
-        <v>-0.04018509761924732</v>
+        <v>-0.0401850976192473</v>
       </c>
       <c r="U69" t="inlineStr">
         <is>
@@ -10601,19 +10613,19 @@
         <v>1.296574206191168</v>
       </c>
       <c r="P70" t="n">
-        <v>-0.3969813378884908</v>
+        <v>-0.3969813378884907</v>
       </c>
       <c r="Q70" t="n">
         <v>-0.3712324202807319</v>
       </c>
       <c r="R70" t="n">
-        <v>-0.02574891760775888</v>
+        <v>-0.0257489176077588</v>
       </c>
       <c r="S70" t="n">
-        <v>-0.04081197882338888</v>
+        <v>-0.0408119788233888</v>
       </c>
       <c r="T70" t="n">
-        <v>-0.04594307391703356</v>
+        <v>-0.0459430739170335</v>
       </c>
       <c r="U70" t="inlineStr">
         <is>
@@ -10821,7 +10833,7 @@
         <v>16.329</v>
       </c>
       <c r="AJ71" t="n">
-        <v>92.58300000000001</v>
+        <v>92.583</v>
       </c>
       <c r="AK71" t="n">
         <v>0</v>
@@ -10899,13 +10911,13 @@
         <v>-0.09146955421090169</v>
       </c>
       <c r="R72" t="n">
-        <v>0.001282960254139598</v>
+        <v>0.0012829602541395</v>
       </c>
       <c r="S72" t="n">
-        <v>0.008886413911057989</v>
+        <v>0.0088864139110579</v>
       </c>
       <c r="T72" t="n">
-        <v>0.01651845140713303</v>
+        <v>0.016518451407133</v>
       </c>
       <c r="U72" t="inlineStr">
         <is>
@@ -11042,16 +11054,16 @@
         <v>-0.1986627672208634</v>
       </c>
       <c r="Q73" t="n">
-        <v>-0.07458934626741741</v>
+        <v>-0.07458934626741739</v>
       </c>
       <c r="R73" t="n">
-        <v>-0.124073420953446</v>
+        <v>-0.1240734209534459</v>
       </c>
       <c r="S73" t="n">
-        <v>-0.08172192532351477</v>
+        <v>-0.0817219253235147</v>
       </c>
       <c r="T73" t="n">
-        <v>-0.03213790003555367</v>
+        <v>-0.0321379000355536</v>
       </c>
       <c r="U73" t="inlineStr">
         <is>
@@ -11194,10 +11206,10 @@
         <v>-0.0337716413234817</v>
       </c>
       <c r="S74" t="n">
-        <v>-0.03779790800102334</v>
+        <v>-0.0377979080010233</v>
       </c>
       <c r="T74" t="n">
-        <v>-0.0498603171619097</v>
+        <v>-0.0498603171619096</v>
       </c>
       <c r="U74" t="inlineStr">
         <is>
@@ -11331,19 +11343,19 @@
         <v>1.20745786778005</v>
       </c>
       <c r="P75" t="n">
-        <v>-0.04918992523716526</v>
+        <v>-0.0491899252371652</v>
       </c>
       <c r="Q75" t="n">
-        <v>-0.002476350378548896</v>
+        <v>-0.0024763503785488</v>
       </c>
       <c r="R75" t="n">
-        <v>-0.04671357485861636</v>
+        <v>-0.0467135748586163</v>
       </c>
       <c r="S75" t="n">
-        <v>-0.05146954958609007</v>
+        <v>-0.05146954958609</v>
       </c>
       <c r="T75" t="n">
-        <v>-0.04979578161098822</v>
+        <v>-0.0497957816109882</v>
       </c>
       <c r="U75" t="inlineStr">
         <is>
@@ -11486,7 +11498,7 @@
         <v>-0.0238995398730405</v>
       </c>
       <c r="S76" t="n">
-        <v>-0.03399371352818775</v>
+        <v>-0.0339937135281877</v>
       </c>
       <c r="T76" t="n">
         <v>-0.07709330811998499</v>
@@ -11623,19 +11635,19 @@
         <v>1.154899945711243</v>
       </c>
       <c r="P77" t="n">
-        <v>-0.1906615946628634</v>
+        <v>-0.1906615946628633</v>
       </c>
       <c r="Q77" t="n">
-        <v>-0.2451463397457728</v>
+        <v>-0.2451463397457727</v>
       </c>
       <c r="R77" t="n">
         <v>0.0544847450829094</v>
       </c>
       <c r="S77" t="n">
-        <v>0.07617478882841211</v>
+        <v>0.0761747888284121</v>
       </c>
       <c r="T77" t="n">
-        <v>0.1081731766624207</v>
+        <v>0.1081731766624206</v>
       </c>
       <c r="U77" t="inlineStr">
         <is>
@@ -11703,7 +11715,7 @@
         <v>217</v>
       </c>
       <c r="AL77" t="n">
-        <v>23.10900000000009</v>
+        <v>23.1090000000001</v>
       </c>
       <c r="AM77" t="n">
         <v>-10753.257</v>
@@ -11775,10 +11787,10 @@
         <v>1.129502847612775</v>
       </c>
       <c r="R78" t="n">
-        <v>-0.1987729035799415</v>
+        <v>-0.1987729035799414</v>
       </c>
       <c r="S78" t="n">
-        <v>-0.0009894930271550084</v>
+        <v>-0.000989493027155</v>
       </c>
       <c r="T78" t="n">
         <v>0.328041528335933</v>
@@ -11837,7 +11849,7 @@
         <v>69.36499999999999</v>
       </c>
       <c r="AH78" t="n">
-        <v>-968.2829999999999</v>
+        <v>-968.283</v>
       </c>
       <c r="AI78" t="n">
         <v>-17562.534</v>
@@ -12067,13 +12079,13 @@
         <v>-0.1856721987206606</v>
       </c>
       <c r="R80" t="n">
-        <v>-0.01192555654418206</v>
+        <v>-0.011925556544182</v>
       </c>
       <c r="S80" t="n">
-        <v>-0.02569536440434408</v>
+        <v>-0.025695364404344</v>
       </c>
       <c r="T80" t="n">
-        <v>-0.03267622221472419</v>
+        <v>-0.0326762222147241</v>
       </c>
       <c r="U80" t="inlineStr">
         <is>
@@ -12216,10 +12228,10 @@
         <v>-0.0164712329819181</v>
       </c>
       <c r="S81" t="n">
-        <v>-0.02100156041681162</v>
+        <v>-0.0210015604168116</v>
       </c>
       <c r="T81" t="n">
-        <v>-0.0242133394541208</v>
+        <v>-0.0242133394541207</v>
       </c>
       <c r="U81" t="inlineStr">
         <is>
@@ -12359,7 +12371,7 @@
         <v>-5.363531062892289</v>
       </c>
       <c r="R82" t="n">
-        <v>-0.01363398268947336</v>
+        <v>-0.0136339826894733</v>
       </c>
       <c r="S82" t="n">
         <v>-0.2907488373747613</v>
@@ -12469,7 +12481,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>91.19999694824219</v>
+        <v>91.1999969482422</v>
       </c>
       <c r="G83" t="n">
         <v>88.19500007629395</v>
@@ -12499,7 +12511,7 @@
         <v>2.177625421066826</v>
       </c>
       <c r="P83" t="n">
-        <v>0.2123990647558998</v>
+        <v>0.2123990647558997</v>
       </c>
       <c r="Q83" t="n">
         <v>-0.5076708260419354</v>
@@ -12570,7 +12582,7 @@
         <v>-0.6099999999999999</v>
       </c>
       <c r="AI83" t="n">
-        <v>-0.1099999999999959</v>
+        <v>-0.1099999999999958</v>
       </c>
       <c r="AJ83" t="n">
         <v>-162.158</v>
@@ -12651,13 +12663,13 @@
         <v>-0.4439444866145415</v>
       </c>
       <c r="R84" t="n">
-        <v>0.03872435310118477</v>
+        <v>0.0387243531011847</v>
       </c>
       <c r="S84" t="n">
-        <v>-0.05912278007257576</v>
+        <v>-0.0591227800725757</v>
       </c>
       <c r="T84" t="n">
-        <v>-0.1110358990224679</v>
+        <v>-0.1110358990224678</v>
       </c>
       <c r="U84" t="inlineStr">
         <is>
@@ -12791,10 +12803,10 @@
         <v>1.765449038313258</v>
       </c>
       <c r="P85" t="n">
-        <v>-0.01101717058839213</v>
+        <v>-0.0110171705883921</v>
       </c>
       <c r="Q85" t="n">
-        <v>-0.1306607051435067</v>
+        <v>-0.1306607051435066</v>
       </c>
       <c r="R85" t="n">
         <v>0.1196435345551145</v>
@@ -12943,13 +12955,13 @@
         <v>-0.1123354443014818</v>
       </c>
       <c r="R86" t="n">
-        <v>-0.04051335372012838</v>
+        <v>-0.0405133537201283</v>
       </c>
       <c r="S86" t="n">
-        <v>-0.03457648132944026</v>
+        <v>-0.0345764813294402</v>
       </c>
       <c r="T86" t="n">
-        <v>-0.01563513989971912</v>
+        <v>-0.0156351398997191</v>
       </c>
       <c r="U86" t="inlineStr">
         <is>
@@ -13089,13 +13101,13 @@
         <v>-0.4737895295564234</v>
       </c>
       <c r="R87" t="n">
-        <v>0.09584392774808825</v>
+        <v>0.0958439277480882</v>
       </c>
       <c r="S87" t="n">
-        <v>0.02728843580169615</v>
+        <v>0.0272884358016961</v>
       </c>
       <c r="T87" t="n">
-        <v>-0.07713103353992135</v>
+        <v>-0.0771310335399213</v>
       </c>
       <c r="U87" t="inlineStr">
         <is>
@@ -13235,13 +13247,13 @@
         <v>-0.743714900294794</v>
       </c>
       <c r="R88" t="n">
-        <v>-0.02643913548484633</v>
+        <v>-0.0264391354848463</v>
       </c>
       <c r="S88" t="n">
-        <v>0.01491913176775916</v>
+        <v>0.0149191317677591</v>
       </c>
       <c r="T88" t="n">
-        <v>0.08019645146493393</v>
+        <v>0.0801964514649339</v>
       </c>
       <c r="U88" t="inlineStr">
         <is>
@@ -13384,10 +13396,10 @@
         <v>-0.0237896889531391</v>
       </c>
       <c r="S89" t="n">
-        <v>-0.02015056001327488</v>
+        <v>-0.0201505600132748</v>
       </c>
       <c r="T89" t="n">
-        <v>-0.01893743788720503</v>
+        <v>-0.018937437887205</v>
       </c>
       <c r="U89" t="inlineStr">
         <is>
@@ -13527,13 +13539,13 @@
         <v>-0.4728125493370557</v>
       </c>
       <c r="R90" t="n">
-        <v>0.01707051292762657</v>
+        <v>0.0170705129276265</v>
       </c>
       <c r="S90" t="n">
-        <v>-0.008125595359321447</v>
+        <v>-0.0081255953593214</v>
       </c>
       <c r="T90" t="n">
-        <v>-0.04579682607908009</v>
+        <v>-0.04579682607908</v>
       </c>
       <c r="U90" t="inlineStr">
         <is>
@@ -13667,19 +13679,19 @@
         <v>1.408547666134687</v>
       </c>
       <c r="P91" t="n">
-        <v>0.06031079270208295</v>
+        <v>0.0603107927020829</v>
       </c>
       <c r="Q91" t="n">
-        <v>-0.04279694478817513</v>
+        <v>-0.0427969447881751</v>
       </c>
       <c r="R91" t="n">
-        <v>0.1031077374902581</v>
+        <v>0.103107737490258</v>
       </c>
       <c r="S91" t="n">
         <v>0.1063850257404778</v>
       </c>
       <c r="T91" t="n">
-        <v>0.1495316370166237</v>
+        <v>0.1495316370166236</v>
       </c>
       <c r="U91" t="inlineStr">
         <is>
@@ -13819,13 +13831,13 @@
         <v>-0.5157658515448551</v>
       </c>
       <c r="R92" t="n">
-        <v>0.07312005209358485</v>
+        <v>0.0731200520935848</v>
       </c>
       <c r="S92" t="n">
-        <v>-0.00820024988032253</v>
+        <v>-0.0082002498803225</v>
       </c>
       <c r="T92" t="n">
-        <v>0.002874242309343744</v>
+        <v>0.0028742423093437</v>
       </c>
       <c r="U92" t="inlineStr">
         <is>
@@ -13965,13 +13977,13 @@
         <v>-0.3687022076974349</v>
       </c>
       <c r="R93" t="n">
-        <v>-0.05992403875488267</v>
+        <v>-0.0599240387548826</v>
       </c>
       <c r="S93" t="n">
-        <v>-0.05288275182624186</v>
+        <v>-0.0528827518262418</v>
       </c>
       <c r="T93" t="n">
-        <v>-0.02698991051106081</v>
+        <v>-0.0269899105110608</v>
       </c>
       <c r="U93" t="inlineStr">
         <is>
@@ -14224,7 +14236,7 @@
         <v>24.45000076293945</v>
       </c>
       <c r="G95" t="n">
-        <v>24.59500007629395</v>
+        <v>24.59500007629394</v>
       </c>
       <c r="H95" t="b">
         <v>0</v>
@@ -14251,16 +14263,16 @@
         <v>1.342068942918894</v>
       </c>
       <c r="P95" t="n">
-        <v>-0.05474978994614332</v>
+        <v>-0.0547497899461433</v>
       </c>
       <c r="Q95" t="n">
-        <v>-0.1191121758885341</v>
+        <v>-0.119112175888534</v>
       </c>
       <c r="R95" t="n">
-        <v>0.06436238594239073</v>
+        <v>0.0643623859423907</v>
       </c>
       <c r="S95" t="n">
-        <v>0.08234051890757801</v>
+        <v>0.082340518907578</v>
       </c>
       <c r="T95" t="n">
         <v>0.1061037370642961</v>
@@ -14403,13 +14415,13 @@
         <v>-0.6615022060536935</v>
       </c>
       <c r="R96" t="n">
-        <v>0.04815228090181711</v>
+        <v>0.0481522809018171</v>
       </c>
       <c r="S96" t="n">
-        <v>0.0001946720350322062</v>
+        <v>0.0001946720350322</v>
       </c>
       <c r="T96" t="n">
-        <v>-0.1072661761966756</v>
+        <v>-0.1072661761966755</v>
       </c>
       <c r="U96" t="inlineStr">
         <is>
@@ -14692,16 +14704,16 @@
         <v>-0.4693326259662189</v>
       </c>
       <c r="Q98" t="n">
-        <v>-0.4407415447034692</v>
+        <v>-0.4407415447034691</v>
       </c>
       <c r="R98" t="n">
-        <v>-0.02859108126274978</v>
+        <v>-0.0285910812627497</v>
       </c>
       <c r="S98" t="n">
-        <v>-0.03049073835550409</v>
+        <v>-0.030490738355504</v>
       </c>
       <c r="T98" t="n">
-        <v>-0.02975553039293743</v>
+        <v>-0.0297555303929374</v>
       </c>
       <c r="U98" t="inlineStr">
         <is>
@@ -14838,7 +14850,7 @@
         <v>-0.4990972135188372</v>
       </c>
       <c r="Q99" t="n">
-        <v>0.348008371068298</v>
+        <v>0.3480083710682979</v>
       </c>
       <c r="R99" t="n">
         <v>-0.8471055845871351</v>
@@ -14993,7 +15005,7 @@
         <v>0.18967779672813</v>
       </c>
       <c r="T100" t="n">
-        <v>0.157234860136511</v>
+        <v>0.1572348601365109</v>
       </c>
       <c r="U100" t="inlineStr">
         <is>
@@ -15127,19 +15139,19 @@
         <v>1.263202639796775</v>
       </c>
       <c r="P101" t="n">
-        <v>0.2764584105717312</v>
+        <v>0.2764584105717311</v>
       </c>
       <c r="Q101" t="n">
         <v>0.3104349203868266</v>
       </c>
       <c r="R101" t="n">
-        <v>-0.03397650981509548</v>
+        <v>-0.0339765098150954</v>
       </c>
       <c r="S101" t="n">
-        <v>-0.01014455492987565</v>
+        <v>-0.0101445549298756</v>
       </c>
       <c r="T101" t="n">
-        <v>0.05463310839961222</v>
+        <v>0.0546331083996122</v>
       </c>
       <c r="U101" t="inlineStr">
         <is>
@@ -15246,7 +15258,7 @@
         <v>25.45000076293945</v>
       </c>
       <c r="G102" t="n">
-        <v>25.34500007629395</v>
+        <v>25.34500007629394</v>
       </c>
       <c r="H102" t="b">
         <v>1</v>
@@ -15276,16 +15288,16 @@
         <v>0.1707121487796357</v>
       </c>
       <c r="Q102" t="n">
-        <v>0.1591224805118085</v>
+        <v>0.1591224805118084</v>
       </c>
       <c r="R102" t="n">
-        <v>0.01158966826782723</v>
+        <v>0.0115896682678272</v>
       </c>
       <c r="S102" t="n">
         <v>0.0171764069228808</v>
       </c>
       <c r="T102" t="n">
-        <v>0.01219919491019639</v>
+        <v>0.0121991949101963</v>
       </c>
       <c r="U102" t="inlineStr">
         <is>
@@ -15419,19 +15431,19 @@
         <v>1.237473806055042</v>
       </c>
       <c r="P103" t="n">
-        <v>0.01922610337012998</v>
+        <v>0.0192261033701299</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.005173869868034567</v>
+        <v>0.0051738698680345</v>
       </c>
       <c r="R103" t="n">
-        <v>0.01405223350209541</v>
+        <v>0.0140522335020954</v>
       </c>
       <c r="S103" t="n">
-        <v>-0.002638757207512808</v>
+        <v>-0.0026387572075128</v>
       </c>
       <c r="T103" t="n">
-        <v>-0.02907193540401273</v>
+        <v>-0.0290719354040127</v>
       </c>
       <c r="U103" t="inlineStr">
         <is>
@@ -15577,7 +15589,7 @@
         <v>-0.1395077610149973</v>
       </c>
       <c r="T104" t="n">
-        <v>-0.01798959408196454</v>
+        <v>-0.0179895940819645</v>
       </c>
       <c r="U104" t="inlineStr">
         <is>
@@ -15717,13 +15729,13 @@
         <v>-0.5815018965148691</v>
       </c>
       <c r="R105" t="n">
-        <v>0.000720587542581308</v>
+        <v>0.0007205875425812999</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.02455030479634046</v>
+        <v>-0.0245503047963404</v>
       </c>
       <c r="T105" t="n">
-        <v>-0.04417307408505444</v>
+        <v>-0.0441730740850544</v>
       </c>
       <c r="U105" t="inlineStr">
         <is>
@@ -15863,7 +15875,7 @@
         <v>-0.3232757569286884</v>
       </c>
       <c r="R106" t="n">
-        <v>-0.08530183716053141</v>
+        <v>-0.0853018371605314</v>
       </c>
       <c r="S106" t="n">
         <v>-0.1043928856295968</v>
@@ -16000,22 +16012,22 @@
         <v>187965.075</v>
       </c>
       <c r="O107" t="n">
-        <v>0.9824689748708401</v>
+        <v>0.98246897487084</v>
       </c>
       <c r="P107" t="n">
-        <v>-0.09454941843869946</v>
+        <v>-0.09454941843869941</v>
       </c>
       <c r="Q107" t="n">
         <v>-0.1212234067730133</v>
       </c>
       <c r="R107" t="n">
-        <v>0.02667398833431388</v>
+        <v>0.0266739883343138</v>
       </c>
       <c r="S107" t="n">
-        <v>0.02905501884558828</v>
+        <v>0.0290550188455882</v>
       </c>
       <c r="T107" t="n">
-        <v>0.02210217752794122</v>
+        <v>0.0221021775279412</v>
       </c>
       <c r="U107" t="inlineStr">
         <is>
@@ -16146,7 +16158,7 @@
         <v>40160.625</v>
       </c>
       <c r="O108" t="n">
-        <v>0.9779115046249821</v>
+        <v>0.977911504624982</v>
       </c>
       <c r="P108" t="n">
         <v>-0.441286785851446</v>
@@ -16161,7 +16173,7 @@
         <v>0.1035884382351014</v>
       </c>
       <c r="T108" t="n">
-        <v>0.07736743790408696</v>
+        <v>0.0773674379040869</v>
       </c>
       <c r="U108" t="inlineStr">
         <is>
@@ -16301,13 +16313,13 @@
         <v>0.8948839590163155</v>
       </c>
       <c r="R109" t="n">
-        <v>-0.07128709944504064</v>
+        <v>-0.07128709944504059</v>
       </c>
       <c r="S109" t="n">
-        <v>0.03238110729627142</v>
+        <v>0.0323811072962714</v>
       </c>
       <c r="T109" t="n">
-        <v>0.2174316578102309</v>
+        <v>0.2174316578102308</v>
       </c>
       <c r="U109" t="inlineStr">
         <is>
@@ -16596,7 +16608,7 @@
         <v>-1.339939434261042</v>
       </c>
       <c r="S111" t="n">
-        <v>-0.9898732307566265</v>
+        <v>-0.9898732307566264</v>
       </c>
       <c r="T111" t="n">
         <v>-0.2736483963386789</v>
@@ -16852,7 +16864,7 @@
         <v>9.5</v>
       </c>
       <c r="G113" t="n">
-        <v>9.430000114440919</v>
+        <v>9.43000011444092</v>
       </c>
       <c r="H113" t="b">
         <v>1</v>
@@ -16879,19 +16891,19 @@
         <v>1.354523549746821</v>
       </c>
       <c r="P113" t="n">
-        <v>0.002306052593366914</v>
+        <v>0.0023060525933669</v>
       </c>
       <c r="Q113" t="n">
         <v>-0.0424829608481905</v>
       </c>
       <c r="R113" t="n">
-        <v>0.04478901344155742</v>
+        <v>0.0447890134415574</v>
       </c>
       <c r="S113" t="n">
-        <v>0.05111862856519004</v>
+        <v>0.05111862856519</v>
       </c>
       <c r="T113" t="n">
-        <v>0.04957722191631726</v>
+        <v>0.0495772219163172</v>
       </c>
       <c r="U113" t="inlineStr">
         <is>
@@ -17031,10 +17043,10 @@
         <v>0.5752795574138145</v>
       </c>
       <c r="R114" t="n">
-        <v>0.004936610062827862</v>
+        <v>0.0049366100628278</v>
       </c>
       <c r="S114" t="n">
-        <v>0.02642087228851897</v>
+        <v>0.0264208722885189</v>
       </c>
       <c r="T114" t="n">
         <v>0.1265021754495792</v>
@@ -17320,16 +17332,16 @@
         <v>-0.309748190721681</v>
       </c>
       <c r="Q116" t="n">
-        <v>-0.293916409985769</v>
+        <v>-0.2939164099857689</v>
       </c>
       <c r="R116" t="n">
-        <v>-0.01583178073591207</v>
+        <v>-0.015831780735912</v>
       </c>
       <c r="S116" t="n">
-        <v>-0.03729606517484407</v>
+        <v>-0.037296065174844</v>
       </c>
       <c r="T116" t="n">
-        <v>-0.04384085346549482</v>
+        <v>-0.0438408534654948</v>
       </c>
       <c r="U116" t="inlineStr">
         <is>
@@ -17445,7 +17457,7 @@
         <v>50.39162483234158</v>
       </c>
       <c r="J117" t="n">
-        <v>51.89844585490204</v>
+        <v>51.89844585490203</v>
       </c>
       <c r="K117" t="n">
         <v>51.0123427848267</v>
@@ -17463,10 +17475,10 @@
         <v>1.374928472017238</v>
       </c>
       <c r="P117" t="n">
-        <v>0.08156098575179627</v>
+        <v>0.0815609857517962</v>
       </c>
       <c r="Q117" t="n">
-        <v>-0.138800461182581</v>
+        <v>-0.1388004611825809</v>
       </c>
       <c r="R117" t="n">
         <v>0.2203614469343772</v>
@@ -17525,7 +17537,7 @@
         <v>-5</v>
       </c>
       <c r="AF117" t="n">
-        <v>-93.30000000000001</v>
+        <v>-93.3</v>
       </c>
       <c r="AG117" t="n">
         <v>0</v>
@@ -17615,10 +17627,10 @@
         <v>-0.2020503495802263</v>
       </c>
       <c r="R118" t="n">
-        <v>0.03606156835212854</v>
+        <v>0.0360615683521285</v>
       </c>
       <c r="S118" t="n">
-        <v>0.06991265137774288</v>
+        <v>0.0699126513777428</v>
       </c>
       <c r="T118" t="n">
         <v>0.1262341542874416</v>
@@ -17764,10 +17776,10 @@
         <v>0.2126408975401602</v>
       </c>
       <c r="S119" t="n">
-        <v>0.2490948387569815</v>
+        <v>0.2490948387569814</v>
       </c>
       <c r="T119" t="n">
-        <v>0.3096065989534597</v>
+        <v>0.3096065989534596</v>
       </c>
       <c r="U119" t="inlineStr">
         <is>

</xml_diff>